<commit_message>
docs: add Simplified Chinese copy for Telega.in
Fill empty CN columns on the MarketplaceProducts Telega.in row from English, using zh-CN.

Co-authored-by: childfocus.ai <childfocus.ai@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/ToTranslate CN 1 (2)(1).xlsx
+++ b/docs/ToTranslate CN 1 (2)(1).xlsx
@@ -19495,6 +19495,39 @@
           <t>Advertising in Telegram and MAX</t>
         </is>
       </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>Telega.in</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>• 超过 36,000 个经过验证的频道目录，按主题、地理位置和参与程度进行过滤。广告投放过程符合广告标签法规的要求
+• 您可以发布文本、照片、视频和活动链接 - 到网站、产品卡、应用程序和其他资源。频道按主题划分 - 轻松找到任何利基市场的目标受众并专门推广产品，无需额外费用
+• Telegram 和 MAX 中的广告有助于快速获得目标受众的浏览量、关注度和转化率。该帖子对所选频道的所有读者都可见。即使使用 Telegram Premium 也无法隐藏或禁用它
+• 维护展示位置统计数据和活动结果预测</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>Telega.in</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>通过 Telega.in 和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>使用 Telega.in 进行有效的商业广告 | 广告市场 sambad.ru</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>Telegram 和 MAX 中的广告</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: keep MarketplaceProducts brand names and original RU spacing
Restore Russian cells from ToTranslate.xlsx so _x000D_ line breaks match the source. Stop translating retailer brands (Lenta, Magnit, Globus, Dixy, Perekrestok, Auchan, Krasnoe i Beloe) in EN/CN.

Co-authored-by: childfocus.ai <childfocus.ai@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/ToTranslate CN 1 (2)(1).xlsx
+++ b/docs/ToTranslate CN 1 (2)(1).xlsx
@@ -9132,9 +9132,10 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Реклама в 2ГИС: Ваш бизнес найдут те, кто ищет!
-Заявите о себе в самом популярном навигаторе для городов!
-— Показывайтесь на карте 2ГИС, когда пользователи ищут услуги в вашем районе.
+          <t>Реклама в 2ГИС: Ваш бизнес найдут те, кто ищет!_x000D_
+_x000D_
+Заявите о себе в самом популярном навигаторе для городов!_x000D_
+— Показывайтесь на карте 2ГИС, когда пользователи ищут услуги в вашем районе._x000D_
 — Выделяйтесь ярким описанием, фото, акциями и высоким рейтингом.</t>
         </is>
       </c>
@@ -9489,8 +9490,10 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Размещение на телевизионных каналах в отдельно взятых регионах.
- Эффективный способ охватить широкую аудиторию в необходимом городе и создать узнаваемость бренда.
+          <t>Размещение на телевизионных каналах в отдельно взятых регионах._x000D_
+ _x000D_
+ Эффективный способ охватить широкую аудиторию в необходимом городе и создать узнаваемость бренда._x000D_
+ _x000D_
  Реклама на ТВ может оказывать сильное эмоциональное воздействие на зрителей благодаря использованию звука, видео и других элементов. Это может способствовать формированию положительного отношения к бренду и повышению лояльности потребителей</t>
         </is>
       </c>
@@ -9674,7 +9677,8 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Размещение на радиостанциях в рекламные блоки в городах России
+          <t>Размещение на радиостанциях в рекламные блоки в городах России_x000D_
+_x000D_
 Радио имеет самую низкую стоимость по достижению максимального охвата. Наиболее эффективно размещение на радио вместе с другими медиа, благодаря чему достигается максимизация эффективной частоты и запоминаемость бренда</t>
         </is>
       </c>
@@ -9764,9 +9768,10 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Реклама в ПВЗ Wildberries: Вовлекайте клиентов в момент выдачи заказов!
-Ваше предложение увидят тысячи покупателей!
-— Размещайте рекламу в пунктах выдачи заказов, где клиенты проводят время в ожидании посылок.
+          <t>Реклама в ПВЗ Wildberries: Вовлекайте клиентов в момент выдачи заказов!_x000D_
+_x000D_
+Ваше предложение увидят тысячи покупателей!_x000D_
+— Размещайте рекламу в пунктах выдачи заказов, где клиенты проводят время в ожидании посылок._x000D_
 — Превращайте их внимание в продажи, лояльность или узнаваемость бренда.</t>
         </is>
       </c>
@@ -10064,7 +10069,8 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Размещение на радиостанциях в качестве спонсора в радио программах, радио рубриках, проведение конкурсов.
+          <t>Размещение на радиостанциях в качестве спонсора в радио программах, радио рубриках, проведение конкурсов._x000D_
+_x000D_
 Радио имеет самую низкую стоимость по достижению максимального охвата. Наиболее эффективно размещение на радио вместе с другими медиа, благодаря чему достигается максимизация эффективной частоты и запоминаемость бренда</t>
         </is>
       </c>
@@ -10154,8 +10160,10 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Статичная наружная реклама размещается в общественных местах, где её может увидеть большое количество людей. Это позволяет быстро донести информацию до широкой аудитории.
-Регулярное появление одних и тех же рекламных сообщений в определённых местах помогает укрепить позиции бренда в сознании потребителей.
+          <t>Статичная наружная реклама размещается в общественных местах, где её может увидеть большое количество людей. Это позволяет быстро донести информацию до широкой аудитории._x000D_
+_x000D_
+Регулярное появление одних и тех же рекламных сообщений в определённых местах помогает укрепить позиции бренда в сознании потребителей._x000D_
+_x000D_
 Размещение в наружной рекламе позволяет составить навигационную адресную программу, что способствует привлечению аудитории к точкам продаж.</t>
         </is>
       </c>
@@ -10434,8 +10442,10 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Реклама в Триколор является эффективным инструментом для продвижения товаров и услуг. Она позволяет охватить широкую аудиторию и донести информацию до потенциальных клиентов.
-Реклама на платформе Триколор может быть направлена на определённые группы людей с учётом их интересов, возраста, пола и других характеристик. Это позволяет более точно достигать целевой аудитории.
+          <t>Реклама в Триколор является эффективным инструментом для продвижения товаров и услуг. Она позволяет охватить широкую аудиторию и донести информацию до потенциальных клиентов._x000D_
+_x000D_
+Реклама на платформе Триколор может быть направлена на определённые группы людей с учётом их интересов, возраста, пола и других характеристик. Это позволяет более точно достигать целевой аудитории._x000D_
+_x000D_
 Обширная сеть вещания Триколор позволяет охватить аудиторию, которым недоступны стандартные медиа.</t>
         </is>
       </c>
@@ -10960,9 +10970,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Захватите внимание миллионной аудитории с рекламой в метро!
-Массовый охват: Вашу рекламу увидят тысячи потенциальных клиентов ежедневно.
-Долгий контакт: Время в пути — это время вашего бренда в голове у пассажира.
+          <t>Захватите внимание миллионной аудитории с рекламой в метро!_x000D_
+_x000D_
+Массовый охват: Вашу рекламу увидят тысячи потенциальных клиентов ежедневно._x000D_
+_x000D_
+Долгий контакт: Время в пути — это время вашего бренда в голове у пассажира._x000D_
+_x000D_
 Нет конкуренции: В вагоне и на эскалаторе ваш бренд — главный объект внимания.</t>
         </is>
       </c>
@@ -11458,10 +11471,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Реклама на Яндекс Картах: Привлеките клиентов рядом с вами!
-Ваш бизнес заметят тысячи!
-— Показывайтесь на картах, когда пользователи ищут услуги в вашем районе.
-— Выделяйтесь среди конкурентов ярким описанием, фото и акциями.
+          <t>Реклама на Яндекс Картах: Привлеките клиентов рядом с вами!_x000D_
+_x000D_
+Ваш бизнес заметят тысячи!_x000D_
+— Показывайтесь на картах, когда пользователи ищут услуги в вашем районе._x000D_
+— Выделяйтесь среди конкурентов ярким описанием, фото и акциями._x000D_
 — Удобные контакты: кнопка «Позвонить», ссылка на сайт, онлайн-запись.</t>
         </is>
       </c>
@@ -11557,7 +11571,8 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Реклама на приставках Ростелеком является эффективным инструментом для продвижения товаров и услуг. Она позволяет охватить широкую аудиторию и донести информацию до потенциальных клиентов.
+          <t>Реклама на приставках Ростелеком является эффективным инструментом для продвижения товаров и услуг. Она позволяет охватить широкую аудиторию и донести информацию до потенциальных клиентов._x000D_
+_x000D_
 Обширная сеть вещания Ростелекома позволяет охватить аудиторию, которым недоступны стандартные медиа.</t>
         </is>
       </c>
@@ -11761,9 +11776,10 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Реклама в Яндекс Метро: Встречайте клиентов на их ежедневном маршруте!
-Ваш бизнес — на пути тысяч пассажиров!
-— Показывайтесь пользователям при планировании маршрутов в метро.
+          <t>Реклама в Яндекс Метро: Встречайте клиентов на их ежедневном маршруте!_x000D_
+_x000D_
+Ваш бизнес — на пути тысяч пассажиров!_x000D_
+— Показывайтесь пользователям при планировании маршрутов в метро._x000D_
 — Привлекайте аудиторию, которая ищет услуги рядом со станциями.</t>
         </is>
       </c>
@@ -11944,11 +11960,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Сервис по персонализированной рассылки электронных писем потенциальным клиентам или партнерам, с которыми у вас ранее не было предварительного контакта. Основная цель такой рассылки — не моментальная продажа, а установление контакта, инициирование диалога и выстраивание деловых отношений для дальнейшего продвижения продукта или услуги. В отличие от массового имэйл-маркетинга, холодный аутрич отличается высокой степенью персонализации сообщений, направленных на конкретного человека и его бизнес-потребности.
-Персонализация: Каждое письмо составляется с учетом конкретного адресата и его ситуации, а не является шаблонным. 
-Ориентация на диалог: Цель – получить ответ и начать разговор с потенциальным клиентом, а не просто отправить информацию. 
-Целевая аудитория: Письма отправляются людям, которые могут быть заинтересованы в вашем предложении, а не случайным получателям. 
-Отличие от спама: Холодный аутрич не является массовым рассылочным спамом, так как ориентирован на боли и интересы конкретных людей и содержит ценное предложение. 
+          <t>Сервис по персонализированной рассылки электронных писем потенциальным клиентам или партнерам, с которыми у вас ранее не было предварительного контакта. Основная цель такой рассылки — не моментальная продажа, а установление контакта, инициирование диалога и выстраивание деловых отношений для дальнейшего продвижения продукта или услуги. В отличие от массового имэйл-маркетинга, холодный аутрич отличается высокой степенью персонализации сообщений, направленных на конкретного человека и его бизнес-потребности._x000D_
+_x000D_
+Персонализация: Каждое письмо составляется с учетом конкретного адресата и его ситуации, а не является шаблонным. _x000D_
+_x000D_
+Ориентация на диалог: Цель – получить ответ и начать разговор с потенциальным клиентом, а не просто отправить информацию. _x000D_
+_x000D_
+Целевая аудитория: Письма отправляются людям, которые могут быть заинтересованы в вашем предложении, а не случайным получателям. _x000D_
+_x000D_
+Отличие от спама: Холодный аутрич не является массовым рассылочным спамом, так как ориентирован на боли и интересы конкретных людей и содержит ценное предложение. _x000D_
+_x000D_
 Масштабируемость: Это экономически эффективный инструмент для бизнеса любого размера, позволяющий охватить большое количество потенциальных клиентов</t>
         </is>
       </c>
@@ -12158,57 +12179,57 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Red and white</t>
+          <t>Krasnoe i Beloe</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Get closer to customers with advertising in Krasnoe and Beloe stores</t>
+          <t>Get closer to customers with advertising in Krasnoe i Beloe stores</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Red and white</t>
+          <t>Krasnoe i Beloe</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Effective advertising in Red and White and other available media channels and formats. Placement experience, full compliance with legislation. Large selection of advertising tools on the advertising marketplace sambad.ru</t>
+          <t>Effective advertising in Krasnoe i Beloe and other available media channels and formats. Placement experience, full compliance with legislation. Large selection of advertising tools on the advertising marketplace sambad.ru</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Effective advertising in Red and White for business | Advertising marketplace sambad.ru</t>
+          <t>Effective advertising in Krasnoe i Beloe for business | Advertising marketplace sambad.ru</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Your advertising in Red and White</t>
+          <t>Your advertising in Krasnoe i Beloe</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>红酒与白酒</t>
+          <t>Krasnoe i Beloe</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>透过在“红与白”门市投放广告，拉近您与顾客的距离</t>
+          <t>透过在“Krasnoe i Beloe”门市投放广告，拉近您与顾客的距离</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>红与白</t>
+          <t>Krasnoe i Beloe</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>在《红与白》为企业投放高效广告 | 广告交易平台 sambad.ru</t>
+          <t>在《Krasnoe i Beloe》为企业投放高效广告 | 广告交易平台 sambad.ru</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>您的广告将出现在《红白报》上</t>
+          <t>您的广告将出现在Krasnoe i Beloe上</t>
         </is>
       </c>
     </row>
@@ -12220,11 +12241,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Avito — крупнейшая в России и одна из самых популярных в мире онлайн-площадок объявлений. Это универсальный цифровой рынок, где частные лица и компании могут:
-Продавать и покупать: Практически любые новые и б/у товары (от одежды и электроники до автомобилей и запчастей).
-Предлагать и искать услуги: От ремонта и переездов до ИТ и красоты.
-Снимать/сдавать и продавать/покупать недвижимость.
-Искать работу или сотрудников.
+          <t>Avito — крупнейшая в России и одна из самых популярных в мире онлайн-площадок объявлений. Это универсальный цифровой рынок, где частные лица и компании могут:_x000D_
+_x000D_
+Продавать и покупать: Практически любые новые и б/у товары (от одежды и электроники до автомобилей и запчастей)._x000D_
+_x000D_
+Предлагать и искать услуги: От ремонта и переездов до ИТ и красоты._x000D_
+_x000D_
+Снимать/сдавать и продавать/покупать недвижимость._x000D_
+_x000D_
+Искать работу или сотрудников._x000D_
+_x000D_
 Размещать объявления о животных.</t>
         </is>
       </c>
@@ -12411,27 +12437,27 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>家乐福</t>
+          <t>Auchan</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>透过在阿尚（Auchan）门市投放广告，拉近与顾客的距离</t>
+          <t>透过在Auchan门市投放广告，拉近与顾客的距离</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>家乐福</t>
+          <t>Auchan</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>针对企业的阿尚（Auchan）有效广告 | 广告交易平台 sambad.ru</t>
+          <t>针对企业的Auchan有效广告 | 广告交易平台 sambad.ru</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>您的广告将出现在阿尚</t>
+          <t>您的广告将出现在Auchan</t>
         </is>
       </c>
     </row>
@@ -12468,7 +12494,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Lenta</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -12478,22 +12504,22 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Ribbon</t>
+          <t>Lenta</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Effective advertising in Tape and other available media channels and formats. Placement experience, full compliance with legislation. Large selection of advertising tools on the advertising marketplace sambad.ru</t>
+          <t>Effective advertising in Lenta and other available media channels and formats. Placement experience, full compliance with legislation. Large selection of advertising tools on the advertising marketplace sambad.ru</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Effective advertising in Feed for business | Advertising marketplace sambad.ru</t>
+          <t>Effective advertising in Lenta for business | Advertising marketplace sambad.ru</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Your advertising in Feed</t>
+          <t>Your advertising in Lenta</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -12503,7 +12529,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>透过在伦塔（Lenta）门市投放广告，拉近与顾客的距离</t>
+          <t>透过在Lenta门市投放广告，拉近与顾客的距离</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -12878,7 +12904,8 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Крупнейший в России онлайн кинотеатр с аудиторией более 70 млн человек.
+          <t>Крупнейший в России онлайн кинотеатр с аудиторией более 70 млн человек._x000D_
+_x000D_
 Подходит компаниям, которые хотят значительно увеличить знание о своем продукте</t>
         </is>
       </c>
@@ -13206,7 +13233,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Yandex market</t>
+          <t>Yandex Market</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -13216,7 +13243,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Yandex market</t>
+          <t>Yandex Market</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -13293,7 +13320,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>wildberries</t>
+          <t>Wildberries</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -13303,7 +13330,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>wildberries</t>
+          <t>Wildberries</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -13562,8 +13589,10 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Размещение на телевизионных каналах сразу на всей территории России.
- Эффективный способ охватить широкую аудиторию и создать узнаваемость бренда.
+          <t>Размещение на телевизионных каналах сразу на всей территории России._x000D_
+ _x000D_
+ Эффективный способ охватить широкую аудиторию и создать узнаваемость бренда._x000D_
+ _x000D_
  Реклама на ТВ может оказывать сильное эмоциональное воздействие на зрителей благодаря использованию звука, видео и других элементов. Это может способствовать формированию положительного отношения к бренду и повышению лояльности потребителей</t>
         </is>
       </c>
@@ -13881,7 +13910,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Globe</t>
+          <t>Globus</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -13891,12 +13920,12 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Globe</t>
+          <t>Globus</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Effective advertising in Globe and other available media channels and formats. Placement experience, full compliance with legislation. Large selection of advertising tools on the advertising marketplace sambad.ru</t>
+          <t>Effective advertising in Globus and other available media channels and formats. Placement experience, full compliance with legislation. Large selection of advertising tools on the advertising marketplace sambad.ru</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -14146,7 +14175,8 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Размещение на радио в интернете. В процессе прослушивания прерывается эфир и подставляется реклама.
+          <t>Размещение на радио в интернете. В процессе прослушивания прерывается эфир и подставляется реклама._x000D_
+_x000D_
 Радио имеет самую низкую стоимость по достижению максимального охвата. Наиболее эффективно размещение на радио вместе с другими медиа, благодаря чему достигается максимизация эффективной частоты и запоминаемость бренда</t>
         </is>
       </c>
@@ -14323,7 +14353,8 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Размещение на телевизионных каналах сразу на всей территории России. Выходы в наиболее премиальных местах рекламных блоков, что гарантирует более качественный контакт с аудиторией.
+          <t>Размещение на телевизионных каналах сразу на всей территории России. Выходы в наиболее премиальных местах рекламных блоков, что гарантирует более качественный контакт с аудиторией._x000D_
+ _x000D_
  Реклама на ТВ может оказывать сильное эмоциональное воздействие на зрителей благодаря использованию звука, видео и других элементов. Это может способствовать формированию положительного отношения к бренду и повышению лояльности потребителей</t>
         </is>
       </c>
@@ -14854,47 +14885,47 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Dixie</t>
+          <t>Dixy</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Get closer to customers with advertising in Dixie stores</t>
+          <t>Get closer to customers with advertising in Dixy stores</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Dixie</t>
+          <t>Dixy</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Effective advertising in Dixie and other available media channels and formats. Placement experience, full compliance with legislation. Large selection of advertising tools on the advertising marketplace sambad.ru</t>
+          <t>Effective advertising in Dixy and other available media channels and formats. Placement experience, full compliance with legislation. Large selection of advertising tools on the advertising marketplace sambad.ru</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Effective advertising in Dixie for business | Advertising marketplace sambad.ru</t>
+          <t>Effective advertising in Dixy for business | Advertising marketplace sambad.ru</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Your advertising in Dixie</t>
+          <t>Your advertising in Dixy</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>迪克西</t>
+          <t>Dixy</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>透过在迪克西（Dixy）门市投放广告，拉近与顾客的距离</t>
+          <t>透过在Dixy门市投放广告，拉近与顾客的距离</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>迪克西</t>
+          <t>Dixy</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -15398,7 +15429,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Crossroads</t>
+          <t>Perekrestok</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -15408,7 +15439,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Crossroads</t>
+          <t>Perekrestok</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -15428,12 +15459,12 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>佩雷克罗斯特</t>
+          <t>Perekrestok</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>透过在“佩雷克雷斯特克”门市投放广告，拉近与顾客的距离</t>
+          <t>透过在“Perekrestok”门市投放广告，拉近与顾客的距离</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
@@ -15448,7 +15479,7 @@
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>您的广告在“佩雷克雷斯特克”</t>
+          <t>您的广告在“Perekrestok”</t>
         </is>
       </c>
     </row>
@@ -15746,7 +15777,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Chancery and office</t>
+          <t>Stationery and office</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -15756,7 +15787,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Chancery and office</t>
+          <t>Stationery and office</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -16126,9 +16157,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Digital наружная реклама размещается в общественных местах, где её может увидеть большое количество людей. Это позволяет быстро донести информацию до широкой аудитории.
-Регулярное появление одних и тех же рекламных сообщений в определённых местах помогает укрепить позиции бренда в сознании потребителей.
-Размещение в наружной рекламе позволяет составить навигационную адресную программу, что способствует привлечению аудитории к точкам продаж.
+          <t>Digital наружная реклама размещается в общественных местах, где её может увидеть большое количество людей. Это позволяет быстро донести информацию до широкой аудитории._x000D_
+_x000D_
+Регулярное появление одних и тех же рекламных сообщений в определённых местах помогает укрепить позиции бренда в сознании потребителей._x000D_
+_x000D_
+Размещение в наружной рекламе позволяет составить навигационную адресную программу, что способствует привлечению аудитории к точкам продаж._x000D_
+_x000D_
 Большие, яркие и динамичные форматы позволят повысить запоминаемость бренда и лучше привлекают внимание</t>
         </is>
       </c>
@@ -16396,9 +16430,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Захватите внимание миллионной аудитории с рекламой в РЖД!
-Массовый охват: Вашу рекламу увидят тысячи потенциальных клиентов ежедневно.
-Долгий контакт: Время в пути — это время вашего бренда в голове у пассажира.
+          <t>Захватите внимание миллионной аудитории с рекламой в РЖД!_x000D_
+_x000D_
+Массовый охват: Вашу рекламу увидят тысячи потенциальных клиентов ежедневно._x000D_
+_x000D_
+Долгий контакт: Время в пути — это время вашего бренда в голове у пассажира._x000D_
+_x000D_
 Нет конкуренции: В вагоне ваш бренд — главный объект внимания.</t>
         </is>
       </c>
@@ -18388,7 +18425,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Magnet</t>
+          <t>Magnit</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -18398,7 +18435,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Magnet</t>
+          <t>Magnit</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -18408,7 +18445,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Effective advertising in Magnet for business | Advertising marketplace sambad.ru</t>
+          <t>Effective advertising in Magnit for business | Advertising marketplace sambad.ru</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -18537,9 +18574,10 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Реклама в Яндекс Навигаторе: Ваш бизнес — на пути клиентов!
-Попадайте в маршруты тысяч пользователей!
-— Показывайте свою точку на карте водителям и пешеходам, которые ищут услуги в реальном времени.
+          <t>Реклама в Яндекс Навигаторе: Ваш бизнес — на пути клиентов!_x000D_
+_x000D_
+Попадайте в маршруты тысяч пользователей!_x000D_
+— Показывайте свою точку на карте водителям и пешеходам, которые ищут услуги в реальном времени._x000D_
 — Выделяйтесь спецпредложениями, когда пользователи прокладывают путь.</t>
         </is>
       </c>
@@ -19436,10 +19474,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>•        Каталог из более чем 36 тысяч верифицированных каналов, фильтр по тематикам, географии и уровню вовлеченности. Процесс размещения рекламы соответствует требованиям законодательства о маркировке рекламы
-•        Можно публиковать текст, фото, видео и активные ссылки — на сайт, карточку товара, приложение и другие ресурсы. Каналы разделены по тематикам — легко находить свою целевую аудиторию в любой нише и продвигать продукт точечно, без лишних затрат
-•        Реклама в Telegram и МАХ помогает быстро получить просмотры, внимание целевой аудитории и конверсии. Пост видят все читатели выбранных каналов. Его нельзя скрыть или отключить даже с Telegram Premium
-•        Ведется статистика размещений и прогноз результатов кампаний</t>
+          <t xml:space="preserve">•        Каталог из более чем 36 тысяч верифицированных каналов, фильтр по тематикам, географии и уровню вовлеченности. Процесс размещения рекламы соответствует требованиям законодательства о маркировке рекламы_x000D_
+•        Можно публиковать текст, фото, видео и активные ссылки — на сайт, карточку товара, приложение и другие ресурсы. Каналы разделены по тематикам — легко находить свою целевую аудиторию в любой нише и продвигать продукт точечно, без лишних затрат_x000D_
+•        Реклама в Telegram и МАХ помогает быстро получить просмотры, внимание целевой аудитории и конверсии. Пост видят все читатели выбранных каналов. Его нельзя скрыть или отключить даже с Telegram Premium_x000D_
+•        Ведется статистика размещений и прогноз результатов кампаний_x000D_
+</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">

</xml_diff>

<commit_message>
Fill empty CN SeoDescription on MarketplaceProducts from English.
Translate missing Simplified Chinese SEO descriptions from en SeoDescription; leave 12 CN-only rows without English empty.

Co-authored-by: childfocus.ai <childfocus.ai@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/ToTranslate CN 1 (2)(1).xlsx
+++ b/docs/ToTranslate CN 1 (2)(1).xlsx
@@ -9210,6 +9210,11 @@
           <t>2GIS</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>在 2GIS 和其他可用媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>2GIS 企业高效广告 | sambad.ru 广告交易平台</t>
@@ -9297,6 +9302,11 @@
           <t>室内静态广告</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>有效的静态室内广告和其他可用的媒体渠道和格式。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q3" t="inlineStr">
         <is>
           <t>企业高效静态室内广告 | sambad.ru 广告交易平台</t>
@@ -9474,6 +9484,11 @@
       <c r="O5" t="inlineStr">
         <is>
           <t>竞争分析</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>针对您的类别进行有效的市场分析并选择可用的媒体渠道和格式。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -9658,6 +9673,11 @@
           <t>推广策略</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>为您的业务提供有效的推广策略以及可用媒体渠道和格式的选择。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>为您的企业量身打造的有效推广策略 | sambad.ru 广告交易平台</t>
@@ -9747,6 +9767,11 @@
       <c r="O8" t="inlineStr">
         <is>
           <t>广播广告</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>在广播和其他可用媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -9846,6 +9871,11 @@
           <t>Wildberries 自取点</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>在 Wildberry 展厅和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q9" t="inlineStr">
         <is>
           <t>企业高效广播赞助广告 | 广告交易平台 sambad.ru</t>
@@ -10139,6 +10169,11 @@
       <c r="O13" t="inlineStr">
         <is>
           <t>广播赞助</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>在广播和其他可用媒体渠道和格式上进行有效的赞助广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -10236,6 +10271,11 @@
           <t>户外广告</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>在广告牌和其他可用媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t>企业高效广告 | 广告交易平台 sambad.ru</t>
@@ -10518,6 +10558,11 @@
           <t>Tricolor</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>在三色和其他可用媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q19" t="inlineStr">
         <is>
           <t>针对企业的高效“三色”广告 | 广告交易平台 sambad.ru</t>
@@ -10605,6 +10650,11 @@
           <t>VOX</t>
         </is>
       </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>通过 VOX 和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q20" t="inlineStr">
         <is>
           <t>针对企业的高效 VOX 广告 | 广告交易平台 sambad.ru</t>
@@ -10747,6 +10797,11 @@
           <t>室内数位广告</t>
         </is>
       </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>有效的数字室内广告和其他可用的媒体渠道和格式。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q23" t="inlineStr">
         <is>
           <t>企业专属高效数位室内广告 | sambad.ru 广告交易平台</t>
@@ -10834,6 +10889,11 @@
           <t>VK</t>
         </is>
       </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>在 VK 和其他可用媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t>企业专属 VK 高效广告 | sambad.ru 广告交易平台</t>
@@ -10919,6 +10979,11 @@
       <c r="O25" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>在 OK 和其他可用的媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -11050,6 +11115,11 @@
           <t>地铁广告</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>在地铁和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q27" t="inlineStr">
         <is>
           <t>针对企业的高效地铁广告 | sambad.ru 广告交易平台</t>
@@ -11137,6 +11207,11 @@
           <t>TG Ads</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>在 TG ADS 和其他可用媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q28" t="inlineStr">
         <is>
           <t>针对企业的高效 TG ADS 广告 | sambad.ru 广告交易平台</t>
@@ -11278,6 +11353,11 @@
           <t>促销页面</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>在促销页面和其他可用的媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q31" t="inlineStr">
         <is>
           <t>企业在推广页面上的高效广告 | sambad.ru 广告交易平台</t>
@@ -11365,6 +11445,11 @@
           <t>Zen</t>
         </is>
       </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>在 ZEN 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q32" t="inlineStr">
         <is>
           <t>企业在 DZEN 上的高效广告 | sambad.ru 广告市场</t>
@@ -11450,6 +11535,11 @@
       <c r="O33" t="inlineStr">
         <is>
           <t>Yandex RYA</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>在 Yandex YAN 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -11552,6 +11642,11 @@
           <t>Yandex 地图</t>
         </is>
       </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>在 Yandex 地图和其他可用媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q34" t="inlineStr">
         <is>
           <t>Yandex 地图上的高效企业广告 | 广告交易平台 sambad.ru</t>
@@ -11643,6 +11738,11 @@
           <t>Rostelecom</t>
         </is>
       </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>在 Rostelecom 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q35" t="inlineStr">
         <is>
           <t>Rostelecom 上的高效企业广告 | 广告交易平台 sambad.ru</t>
@@ -11755,6 +11855,11 @@
       <c r="O37" t="inlineStr">
         <is>
           <t>Digital Alliance</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>在数字联盟和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -11854,6 +11959,11 @@
           <t>Yandex Metro</t>
         </is>
       </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>在 Yandex Metro 和其他可用媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q38" t="inlineStr">
         <is>
           <t>企业在 Yandex Metro 上的高效广告 | sambad.ru 广告市场</t>
@@ -11939,6 +12049,11 @@
       <c r="O39" t="inlineStr">
         <is>
           <t>Pyaterochka</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>在 Pyaterochka 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -12048,6 +12163,11 @@
           <t>Coldy</t>
         </is>
       </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>使用 Coldy 和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q40" t="inlineStr">
         <is>
           <t>透过 Coldy 为企业投放高效广告 | 广告交易平台 sambad.ru</t>
@@ -12135,6 +12255,11 @@
           <t>市场与类别分析</t>
         </is>
       </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>针对您的类别进行有效的市场分析并选择可用的媒体渠道和格式。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q41" t="inlineStr">
         <is>
           <t>您所属类别的高效市场分析 | 广告交易平台 sambad.ru</t>
@@ -12220,6 +12345,11 @@
       <c r="O42" t="inlineStr">
         <is>
           <t>Krasnoe i Beloe</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>在 Krasnoe i Beloe 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -12450,6 +12580,11 @@
           <t>Auchan</t>
         </is>
       </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>在欧尚和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q45" t="inlineStr">
         <is>
           <t>针对企业的Auchan有效广告 | 广告交易平台 sambad.ru</t>
@@ -12537,6 +12672,11 @@
           <t>Lenta</t>
         </is>
       </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>在 Lenta 和其他可用媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q46" t="inlineStr">
         <is>
           <t>针对企业的Lenta有效广告 | 广告交易平台 sambad.ru</t>
@@ -12624,6 +12764,11 @@
           <t>卡片操作</t>
         </is>
       </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>我们将提高您的卡在商店中的转化率，并在所有可用的媒体渠道和格式中投放有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q47" t="inlineStr">
         <is>
           <t>提升您在实体店面的商品页面转换率 | 广告交易平台 sambad.ru</t>
@@ -12711,6 +12856,11 @@
           <t>广播广告</t>
         </is>
       </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>有效的广播广告和其他可用的媒体渠道和格式。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q48" t="inlineStr">
         <is>
           <t>企业高效广播广告 | 广告交易平台 sambad.ru</t>
@@ -12798,6 +12948,11 @@
           <t>电视广告</t>
         </is>
       </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>有效的电视广告和其他可用的媒体渠道和格式。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q49" t="inlineStr">
         <is>
           <t>企业高效电视广告 | 广告交易平台 sambad.ru</t>
@@ -12883,6 +13038,11 @@
       <c r="O50" t="inlineStr">
         <is>
           <t>户外广告创意</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>有效的户外广告创意和其他可用的媒体渠道和格式。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -12976,6 +13136,11 @@
           <t>IVI</t>
         </is>
       </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>在 IVI 和其他可用媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q51" t="inlineStr">
         <is>
           <t>针对企业的高效 IVI 广告 | sambad.ru 广告交易平台</t>
@@ -13189,6 +13354,11 @@
           <t>数位广告创意</t>
         </is>
       </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>有效的数字广告创意和其他可用的媒体渠道和格式。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q54" t="inlineStr">
         <is>
           <t>企业高效数位广告创意 | sambad.ru 广告交易平台</t>
@@ -13276,6 +13446,11 @@
           <t>Yandex Market</t>
         </is>
       </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>在 Yandex Market 和其他可用的媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q55" t="inlineStr">
         <is>
           <t>企业在 Yandex Market 上的高效广告 | sambad.ru 广告交易平台</t>
@@ -13363,6 +13538,11 @@
           <t>Wildberries</t>
         </is>
       </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>在 Wildberry 和其他可用的媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q56" t="inlineStr">
         <is>
           <t>Wildberries 企业高效广告 | sambad.ru 广告交易平台</t>
@@ -13450,6 +13630,11 @@
           <t>Ozon</t>
         </is>
       </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>在 OZON 和其他可用媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q57" t="inlineStr">
         <is>
           <t>OZON 企业高效广告 | sambad.ru 广告交易平台</t>
@@ -13535,6 +13720,11 @@
       <c r="O58" t="inlineStr">
         <is>
           <t>Digital Alliance</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>在数字联盟和其他可用的媒体渠道和格式中进行有效的广告定位。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -13784,6 +13974,11 @@
           <t>RuTube</t>
         </is>
       </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>在 RuTube 和其他可用的媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q62" t="inlineStr">
         <is>
           <t>RuTube 企业高效广告 | sambad.ru 广告交易平台</t>
@@ -13871,6 +14066,11 @@
           <t>A1</t>
         </is>
       </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>利用 A1 和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="R63" t="inlineStr">
         <is>
           <t>自动化处理 Mediascope 与 Admetrix 的报表</t>
@@ -13953,6 +14153,11 @@
           <t>Globus</t>
         </is>
       </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>在 Globus 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q64" t="inlineStr">
         <is>
           <t>Globus 企业高效广告 | sambad.ru 广告交易平台</t>
@@ -14038,6 +14243,11 @@
       <c r="O65" t="inlineStr">
         <is>
           <t>MTS Programmatic</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>在 MTS 程序化和其他可用媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -14247,6 +14457,11 @@
           <t>数位广播</t>
         </is>
       </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>在数字广播和其他可用媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q70" t="inlineStr">
         <is>
           <t>企业专用高效广告 | 广告交易平台 sambad.ru</t>
@@ -14332,6 +14547,11 @@
       <c r="O71" t="inlineStr">
         <is>
           <t>最有效</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>我们将在最有效的业务平台上选择、设置和投放广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -14517,6 +14737,11 @@
           <t>最有效</t>
         </is>
       </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>我们将在最有效的业务平台上选择、设置和投放广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q73" t="inlineStr">
         <is>
           <t>我们将为您挑选、设定并在最有效的商业平台上投放广告 | sambad.ru 广告市场</t>
@@ -14604,6 +14829,11 @@
           <t>最有效</t>
         </is>
       </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>我们将在最有效的业务平台上选择、设置和投放广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q74" t="inlineStr">
         <is>
           <t>我们将为您挑选、设定并在最有效的商业平台上投放广告 | sambad.ru 广告市场</t>
@@ -14691,6 +14921,11 @@
           <t>IT 与数位服务</t>
         </is>
       </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>针对所有可用媒体渠道和格式的 IT 和数字服务的现成广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q75" t="inlineStr">
         <is>
           <t>专为 IT 与数位服务打造的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -14803,6 +15038,11 @@
       <c r="O77" t="inlineStr">
         <is>
           <t>Buzzoola</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>在移动应用程序和其他可用媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -14928,6 +15168,11 @@
           <t>Dixy</t>
         </is>
       </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>在 Dixy 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q79" t="inlineStr">
         <is>
           <t>企业在 Dixy 上的高效广告 | sambad.ru 广告市场</t>
@@ -15015,6 +15260,11 @@
           <t>汽车与交通</t>
         </is>
       </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为汽车和运输类别提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q80" t="inlineStr">
         <is>
           <t>汽车与交通类别的现成广告解决方案 | sambad.ru 广告市场提供丰富的广告工具选择</t>
@@ -15102,6 +15352,11 @@
           <t>安全与防护</t>
         </is>
       </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>针对所有可用媒体渠道和格式的安保和安全服务的现成广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q81" t="inlineStr">
         <is>
           <t>针对安全与保全服务的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -15189,6 +15444,11 @@
           <t>卫生与个人护理</t>
         </is>
       </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为卫生和个人护理产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q82" t="inlineStr">
         <is>
           <t>针对卫生及个人护理产品的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -15276,6 +15536,11 @@
           <t>婴幼儿用品</t>
         </is>
       </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为儿童产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q83" t="inlineStr">
         <is>
           <t>儿童用品的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -15363,6 +15628,11 @@
           <t>宠物用品</t>
         </is>
       </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为宠物产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q84" t="inlineStr">
         <is>
           <t>宠物用品的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -15472,6 +15742,11 @@
           <t>Perekrestok</t>
         </is>
       </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>在 Perekrestok 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q86" t="inlineStr">
         <is>
           <t>在 Perekrestok 为企业投放高效广告 | 广告市场 sambad.ru</t>
@@ -15559,6 +15834,11 @@
           <t>最有效</t>
         </is>
       </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>我们将在最有效的业务平台上选择、设置和投放广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q87" t="inlineStr">
         <is>
           <t>为您的企业精选、设定并投放广告于最具成效的广告平台 | sambad.ru 广告市场</t>
@@ -15646,6 +15926,11 @@
           <t>最有效</t>
         </is>
       </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>我们将在最有效的业务平台上选择、设置和投放广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q88" t="inlineStr">
         <is>
           <t>企业高效广告 | sambad.ru 广告市场</t>
@@ -15733,6 +16018,11 @@
           <t>最有效</t>
         </is>
       </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>我们将在最有效的业务平台上选择、设置和投放广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q89" t="inlineStr">
         <is>
           <t>为您的企业精选、设定并投放广告于最具成效的广告平台 | sambad.ru 广告市场</t>
@@ -15820,6 +16110,11 @@
           <t>文具与办公用品</t>
         </is>
       </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为文具和办公产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q90" t="inlineStr">
         <is>
           <t>针对文具及办公用品的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具选择</t>
@@ -15905,6 +16200,11 @@
       <c r="O91" t="inlineStr">
         <is>
           <t>化妆品与香水</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为化妆品和香水产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
@@ -16051,6 +16351,11 @@
           <t>彩票与博彩</t>
         </is>
       </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>针对所有可用媒体渠道和格式的彩票和投注的现成广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q94" t="inlineStr">
         <is>
           <t>彩票与博彩的现成广告解决方案 | 广告交易平台 sambad.ru 提供丰富的广告工具选择</t>
@@ -16136,6 +16441,11 @@
       <c r="O95" t="inlineStr">
         <is>
           <t>医疗服务</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为医疗服务提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -16237,6 +16547,11 @@
           <t>数位户外广告</t>
         </is>
       </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>在数字广告牌和其他可用媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q96" t="inlineStr">
         <is>
           <t>企业的高效广告 | sambad.ru 广告市场</t>
@@ -16324,6 +16639,11 @@
           <t>房地产及相关交易</t>
         </is>
       </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为房地产市场提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q97" t="inlineStr">
         <is>
           <t>针对房地产市场的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -16409,6 +16729,11 @@
       <c r="O98" t="inlineStr">
         <is>
           <t>教育与职涯</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为教育和职业服务提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
@@ -16510,6 +16835,11 @@
           <t>俄罗斯铁路广告</t>
         </is>
       </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>在俄罗斯铁路和其他可用的媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q99" t="inlineStr">
         <is>
           <t>俄罗斯铁路（RZD）上的高效企业广告 | sambad.ru 广告市场</t>
@@ -16597,6 +16927,11 @@
           <t>Wink</t>
         </is>
       </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>在 WINK 和其他可用的媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q100" t="inlineStr">
         <is>
           <t>企业在 WINK 上的高效广告 | 广告交易平台 sambad.ru</t>
@@ -16684,6 +17019,11 @@
           <t>服饰与配件</t>
         </is>
       </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为服装和配饰提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q101" t="inlineStr">
         <is>
           <t>服饰与配件的现成广告解决方案 | 广告交易平台 sambad.ru 提供丰富多样的广告工具</t>
@@ -16769,6 +17109,11 @@
       <c r="O102" t="inlineStr">
         <is>
           <t>光学与视力</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>在所有可用媒体渠道和格式上为光学和视觉产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -16892,6 +17237,11 @@
           <t>征才</t>
         </is>
       </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>用于所有可用媒体渠道和格式上的搜索和选择服务的现成广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q104" t="inlineStr">
         <is>
           <t>针对人才搜寻与甄选服务的现成广告解决方案 | sambad.ru广告市场提供丰富多样的广告工具</t>
@@ -16979,6 +17329,11 @@
           <t>食品</t>
         </is>
       </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为食品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q105" t="inlineStr">
         <is>
           <t>针对食品的现成广告解决方案 | sambad.ru广告市场提供丰富多样的广告工具</t>
@@ -17066,6 +17421,11 @@
           <t>商品租赁</t>
         </is>
       </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>针对所有可用媒体渠道和格式的租赁服务的现成广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q106" t="inlineStr">
         <is>
           <t>针对商品租赁服务的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -17151,6 +17511,11 @@
       <c r="O107" t="inlineStr">
         <is>
           <t>娱乐与活动</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>针对所有可用媒体渠道和格式的娱乐和活动类别的现成广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -17274,6 +17639,11 @@
           <t>社会、政治与政府服务</t>
         </is>
       </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为社会、政治和政府服务提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q109" t="inlineStr">
         <is>
           <t>针对社会、政治及政府服务的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -17361,6 +17731,11 @@
           <t>运动与休闲活动</t>
         </is>
       </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为运动和户外产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q110" t="inlineStr">
         <is>
           <t>针对运动及户外休闲商品的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -17448,6 +17823,11 @@
           <t>家电与电子产品</t>
         </is>
       </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为技术和电子产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q111" t="inlineStr">
         <is>
           <t>针对家电与电子产品的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -17535,6 +17915,11 @@
           <t>RuStore</t>
         </is>
       </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>在 RuStore 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q112" t="inlineStr">
         <is>
           <t>RuStore 企业高效广告 | 广告市场 sambad.ru</t>
@@ -17622,6 +18007,11 @@
           <t>非酒精饮料</t>
         </is>
       </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为软饮料类别提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q113" t="inlineStr">
         <is>
           <t>无酒精饮料类别的现成广告解决方案 | 广告市场 sambad.ru 提供丰富多样的广告工具</t>
@@ -17707,6 +18097,11 @@
       <c r="O114" t="inlineStr">
         <is>
           <t>建筑与工具</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>适用于所有可用媒体渠道和格式的建筑服务和工具的现成广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -17826,6 +18221,11 @@
           <t>家居用品</t>
         </is>
       </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为家居用品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q116" t="inlineStr">
         <is>
           <t>家居用品的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具选择</t>
@@ -17913,6 +18313,11 @@
           <t>餐饮服务</t>
         </is>
       </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为餐饮服务提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q117" t="inlineStr">
         <is>
           <t>餐饮服务的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具选择</t>
@@ -18000,6 +18405,11 @@
           <t>制药</t>
         </is>
       </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为制药行业提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q118" t="inlineStr">
         <is>
           <t>针对制药产业的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -18120,6 +18530,11 @@
           <t>金融与保险</t>
         </is>
       </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为金融和保险服务提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q120" t="inlineStr">
         <is>
           <t>针对金融服务与保险服务的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -18207,6 +18622,11 @@
           <t>法律服务</t>
         </is>
       </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>针对所有可用媒体渠道和格式的法律服务的现成广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q121" t="inlineStr">
         <is>
           <t>针对法律服务的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -18294,6 +18714,11 @@
           <t>Upravel</t>
         </is>
       </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>利用 Upravel 和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q122" t="inlineStr">
         <is>
           <t>透过 Upravel 为企业提供高效广告 | sambad.ru 广告市场</t>
@@ -18381,6 +18806,11 @@
           <t>Prometheus</t>
         </is>
       </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>使用 Prometheus 和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q123" t="inlineStr">
         <is>
           <t>透过 Prometheus 为企业打造高效广告 | 广告交易平台 sambad.ru</t>
@@ -18468,6 +18898,11 @@
           <t>Magnit</t>
         </is>
       </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>在 Magnit 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q124" t="inlineStr">
         <is>
           <t>在 Magnit 为企业投放高效广告 | 广告交易平台 sambad.ru</t>
@@ -18553,6 +18988,11 @@
       <c r="O125" t="inlineStr">
         <is>
           <t>园艺与菜园</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为园艺类别产品提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
@@ -18652,6 +19092,11 @@
           <t>Yandex 导航</t>
         </is>
       </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>在 Yandex Navigator 和其他可用的媒体渠道和格式中进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q126" t="inlineStr">
         <is>
           <t>企业在 Yandex Navigator 上的高效广告 | 广告交易平台 sambad.ru</t>
@@ -18739,6 +19184,11 @@
           <t>美容与外貌护理服务</t>
         </is>
       </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为美容和美容服务提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q127" t="inlineStr">
         <is>
           <t>针对美容与外貌保养服务的现成广告解决方案 | sambad.ru 广告市场提供丰富多样的广告工具</t>
@@ -18826,6 +19276,11 @@
           <t>V1</t>
         </is>
       </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>利用 V1 和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q128" t="inlineStr">
         <is>
           <t>透过 V1 为企业投放高效广告 | sambad.ru 广告市场</t>
@@ -18940,6 +19395,11 @@
           <t>WOW Bloggers</t>
         </is>
       </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>在 WOW Bloggers 和其他可用的媒体渠道和格式上进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q130" t="inlineStr">
         <is>
           <t>透过 WOW Bloggers 为企业投放高效广告 | 广告交易平台 sambad.ru</t>
@@ -19054,6 +19514,11 @@
           <t>旅游与休闲</t>
         </is>
       </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>在所有可用的媒体渠道和格式上为旅游和休闲市场提供现成的广告解决方案。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q132" t="inlineStr">
         <is>
           <t>旅游与休闲市场的现成广告解决方案 | 广告交易平台 sambad.ru 提供丰富多样的广告工具</t>
@@ -19141,6 +19606,11 @@
           <t>Data Hubble</t>
         </is>
       </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>利用数据和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
+        </is>
+      </c>
       <c r="Q133" t="inlineStr">
         <is>
           <t>透过 Data Hubble 为企业投放高效广告 | 广告交易平台 sambad.ru</t>
@@ -19226,6 +19696,11 @@
       <c r="O134" t="inlineStr">
         <is>
           <t>B1TVP</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>利用 B1TVP 和其他可用的媒体渠道和格式进行有效的广告。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -19453,6 +19928,11 @@
       <c r="O140" t="inlineStr">
         <is>
           <t>Buzzoola</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>在 Buzzoola 和其他可用的媒体渠道和格式中进行有效的广告定位。安置经验，完全遵守法规。广告市场 sambad.ru 上有大量广告工具可供选择</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">

</xml_diff>